<commit_message>
add `replace_invalid_dates` kwarg to Spreadsheet.read
</commit_message>
<xml_diff>
--- a/tests/samples/table.xlsx
+++ b/tests/samples/table.xlsx
@@ -1,28 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.borbely\code\git\msl-io\tests\samples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\J.Borbely\code\msl-io\tests\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABEE5A3-28C7-4681-A7D1-33D1F7BD050C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0511745D-C323-49E3-80AA-1714D741879A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A1" sheetId="1" r:id="rId1"/>
     <sheet name="BH11" sheetId="4" r:id="rId2"/>
     <sheet name="AEX154041" sheetId="2" r:id="rId3"/>
+    <sheet name="BadDates" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="6">
   <si>
     <t>timestamp</t>
   </si>
@@ -38,6 +39,9 @@
   <si>
     <t>uncert2</t>
   </si>
+  <si>
+    <t>Date Acquired</t>
+  </si>
 </sst>
 </file>
 
@@ -47,7 +51,7 @@
     <numFmt numFmtId="164" formatCode="d/mm/yyyy\ h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +185,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -524,10 +539,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -884,14 +903,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="8.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="8.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -908,7 +927,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>43719.588136574072</v>
       </c>
@@ -925,7 +944,7 @@
         <v>7.8999999999999996E-5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>43719.588182870371</v>
       </c>
@@ -942,7 +961,7 @@
         <v>8.2999999999999998E-5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>43719.588229166664</v>
       </c>
@@ -959,7 +978,7 @@
         <v>8.7000000000000001E-5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>43719.588275462964</v>
       </c>
@@ -976,7 +995,7 @@
         <v>1.2E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>43719.588321759256</v>
       </c>
@@ -993,7 +1012,7 @@
         <v>8.7999999999999998E-5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>43719.588368055556</v>
       </c>
@@ -1010,7 +1029,7 @@
         <v>8.5000000000000006E-5</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>43719.588414351849</v>
       </c>
@@ -1027,7 +1046,7 @@
         <v>8.3999999999999995E-5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>43719.588460648149</v>
       </c>
@@ -1044,7 +1063,7 @@
         <v>7.6000000000000004E-5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>43719.588506944441</v>
       </c>
@@ -1061,7 +1080,7 @@
         <v>6.2000000000000003E-5</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>43719.588553240741</v>
       </c>
@@ -1086,14 +1105,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C522F26F-3350-42E8-911C-A1B510332815}">
   <dimension ref="BH11:BL21"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="60" max="60" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="9.265625" bestFit="1" customWidth="1"/>
-    <col min="62" max="64" width="8.59765625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="62" max="64" width="8.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="11" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH11" t="s">
         <v>0</v>
       </c>
@@ -1110,7 +1129,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="12" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH12" s="1">
         <v>43719.588136574072</v>
       </c>
@@ -1127,7 +1146,7 @@
         <v>7.8999999999999996E-5</v>
       </c>
     </row>
-    <row r="13" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="13" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH13" s="1">
         <v>43719.588182870371</v>
       </c>
@@ -1144,7 +1163,7 @@
         <v>8.2999999999999998E-5</v>
       </c>
     </row>
-    <row r="14" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="14" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH14" s="1">
         <v>43719.588229166664</v>
       </c>
@@ -1161,7 +1180,7 @@
         <v>8.7000000000000001E-5</v>
       </c>
     </row>
-    <row r="15" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="15" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH15" s="1">
         <v>43719.588275462964</v>
       </c>
@@ -1178,7 +1197,7 @@
         <v>1.2E-4</v>
       </c>
     </row>
-    <row r="16" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="16" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH16" s="1">
         <v>43719.588321759256</v>
       </c>
@@ -1195,7 +1214,7 @@
         <v>8.7999999999999998E-5</v>
       </c>
     </row>
-    <row r="17" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="17" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH17" s="1">
         <v>43719.588368055556</v>
       </c>
@@ -1212,7 +1231,7 @@
         <v>8.5000000000000006E-5</v>
       </c>
     </row>
-    <row r="18" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="18" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH18" s="1">
         <v>43719.588414351849</v>
       </c>
@@ -1229,7 +1248,7 @@
         <v>8.3999999999999995E-5</v>
       </c>
     </row>
-    <row r="19" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="19" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH19" s="1">
         <v>43719.588460648149</v>
       </c>
@@ -1246,7 +1265,7 @@
         <v>7.6000000000000004E-5</v>
       </c>
     </row>
-    <row r="20" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="20" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH20" s="1">
         <v>43719.588506944441</v>
       </c>
@@ -1263,7 +1282,7 @@
         <v>6.2000000000000003E-5</v>
       </c>
     </row>
-    <row r="21" spans="60:64" x14ac:dyDescent="0.45">
+    <row r="21" spans="60:64" x14ac:dyDescent="0.35">
       <c r="BH21" s="1">
         <v>43719.588553240741</v>
       </c>
@@ -1288,14 +1307,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="AEX154041:AFB154051"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="830" max="830" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="831" max="831" width="9.265625" bestFit="1" customWidth="1"/>
-    <col min="832" max="834" width="8.59765625" bestFit="1" customWidth="1"/>
+    <col min="830" max="830" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="831" max="831" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="832" max="834" width="8.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="154041" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154041" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154041" t="s">
         <v>0</v>
       </c>
@@ -1312,7 +1331,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="154042" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154042" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154042" s="1">
         <v>43719.588136574072</v>
       </c>
@@ -1329,7 +1348,7 @@
         <v>7.8999999999999996E-5</v>
       </c>
     </row>
-    <row r="154043" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154043" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154043" s="1">
         <v>43719.588182870371</v>
       </c>
@@ -1346,7 +1365,7 @@
         <v>8.2999999999999998E-5</v>
       </c>
     </row>
-    <row r="154044" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154044" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154044" s="1">
         <v>43719.588229166664</v>
       </c>
@@ -1363,7 +1382,7 @@
         <v>8.7000000000000001E-5</v>
       </c>
     </row>
-    <row r="154045" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154045" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154045" s="1">
         <v>43719.588275462964</v>
       </c>
@@ -1380,7 +1399,7 @@
         <v>1.2E-4</v>
       </c>
     </row>
-    <row r="154046" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154046" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154046" s="1">
         <v>43719.588321759256</v>
       </c>
@@ -1397,7 +1416,7 @@
         <v>8.7999999999999998E-5</v>
       </c>
     </row>
-    <row r="154047" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154047" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154047" s="1">
         <v>43719.588368055556</v>
       </c>
@@ -1414,7 +1433,7 @@
         <v>8.5000000000000006E-5</v>
       </c>
     </row>
-    <row r="154048" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154048" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154048" s="1">
         <v>43719.588414351849</v>
       </c>
@@ -1431,7 +1450,7 @@
         <v>8.3999999999999995E-5</v>
       </c>
     </row>
-    <row r="154049" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154049" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154049" s="1">
         <v>43719.588460648149</v>
       </c>
@@ -1448,7 +1467,7 @@
         <v>7.6000000000000004E-5</v>
       </c>
     </row>
-    <row r="154050" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154050" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154050" s="1">
         <v>43719.588506944441</v>
       </c>
@@ -1465,7 +1484,7 @@
         <v>6.2000000000000003E-5</v>
       </c>
     </row>
-    <row r="154051" spans="830:834" x14ac:dyDescent="0.45">
+    <row r="154051" spans="830:834" x14ac:dyDescent="0.35">
       <c r="AEX154051" s="1">
         <v>43719.588553240741</v>
       </c>
@@ -1485,4 +1504,38 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F82A60-CDC6-4577-9954-B403FAAB4BCB}">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>44730</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>45566</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>